<commit_message>
Updated Lineux Stealth Bom
Updated Lineux Stealth Bom
</commit_message>
<xml_diff>
--- a/BOM/Lineux Stealth Bom.xlsx
+++ b/BOM/Lineux Stealth Bom.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="86">
   <si>
     <t>Lineux Stealth Bill Of Material</t>
   </si>
@@ -143,6 +143,9 @@
   </si>
   <si>
     <t>Lineux Stealth Tiga Toolhead</t>
+  </si>
+  <si>
+    <t>m2 x 8mm self tap screw</t>
   </si>
   <si>
     <t>m3 x 6mm bhcs</t>
@@ -2425,11 +2428,11 @@
       <c r="Z51" s="4"/>
     </row>
     <row r="52">
-      <c r="A52" s="9" t="s">
-        <v>12</v>
+      <c r="A52" s="18" t="s">
+        <v>44</v>
       </c>
       <c r="B52" s="17">
-        <v>23.0</v>
+        <v>2.0</v>
       </c>
       <c r="C52" s="4"/>
       <c r="D52" s="4"/>
@@ -2458,10 +2461,10 @@
     </row>
     <row r="53">
       <c r="A53" s="9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B53" s="17">
-        <v>5.0</v>
+        <v>23.0</v>
       </c>
       <c r="C53" s="4"/>
       <c r="D53" s="4"/>
@@ -2489,11 +2492,11 @@
       <c r="Z53" s="4"/>
     </row>
     <row r="54">
-      <c r="A54" s="18" t="s">
-        <v>44</v>
+      <c r="A54" s="9" t="s">
+        <v>13</v>
       </c>
       <c r="B54" s="17">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="C54" s="4"/>
       <c r="D54" s="4"/>
@@ -2525,11 +2528,11 @@
         <v>45</v>
       </c>
       <c r="B55" s="17">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="C55" s="4"/>
       <c r="D55" s="4"/>
-      <c r="E55" s="22"/>
+      <c r="E55" s="10"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -2586,7 +2589,7 @@
     </row>
     <row r="57">
       <c r="A57" s="18" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="B57" s="17">
         <v>2.0</v>
@@ -2618,14 +2621,14 @@
     </row>
     <row r="58">
       <c r="A58" s="18" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="B58" s="17">
-        <v>5.0</v>
+        <v>2.0</v>
       </c>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
-      <c r="E58" s="10"/>
+      <c r="E58" s="22"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -2650,10 +2653,10 @@
     </row>
     <row r="59">
       <c r="A59" s="18" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="B59" s="17">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="C59" s="4"/>
       <c r="D59" s="4"/>
@@ -2685,11 +2688,11 @@
         <v>48</v>
       </c>
       <c r="B60" s="17">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="C60" s="4"/>
       <c r="D60" s="4"/>
-      <c r="E60" s="22"/>
+      <c r="E60" s="10"/>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
@@ -2717,7 +2720,7 @@
         <v>49</v>
       </c>
       <c r="B61" s="17">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
@@ -2745,15 +2748,15 @@
       <c r="Z61" s="4"/>
     </row>
     <row r="62">
-      <c r="A62" s="9" t="s">
+      <c r="A62" s="18" t="s">
         <v>50</v>
       </c>
       <c r="B62" s="17">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
-      <c r="E62" s="10"/>
+      <c r="E62" s="22"/>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
       <c r="H62" s="4"/>
@@ -2781,7 +2784,7 @@
         <v>51</v>
       </c>
       <c r="B63" s="17">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
@@ -2848,9 +2851,7 @@
         <v>4.0</v>
       </c>
       <c r="C65" s="4"/>
-      <c r="D65" s="19" t="s">
-        <v>21</v>
-      </c>
+      <c r="D65" s="4"/>
       <c r="E65" s="10"/>
       <c r="F65" s="4"/>
       <c r="G65" s="4"/>
@@ -2876,13 +2877,15 @@
     </row>
     <row r="66">
       <c r="A66" s="9" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="B66" s="17">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="C66" s="4"/>
-      <c r="D66" s="4"/>
+      <c r="D66" s="19" t="s">
+        <v>21</v>
+      </c>
       <c r="E66" s="10"/>
       <c r="F66" s="4"/>
       <c r="G66" s="4"/>
@@ -2908,10 +2911,10 @@
     </row>
     <row r="67">
       <c r="A67" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B67" s="17">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
@@ -2940,15 +2943,13 @@
     </row>
     <row r="68">
       <c r="A68" s="9" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B68" s="17">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="C68" s="4"/>
-      <c r="D68" s="19" t="s">
-        <v>21</v>
-      </c>
+      <c r="D68" s="4"/>
       <c r="E68" s="10"/>
       <c r="F68" s="4"/>
       <c r="G68" s="4"/>
@@ -2973,17 +2974,17 @@
       <c r="Z68" s="4"/>
     </row>
     <row r="69">
-      <c r="A69" s="18" t="s">
-        <v>54</v>
+      <c r="A69" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="B69" s="17">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="C69" s="4"/>
-      <c r="D69" s="19"/>
-      <c r="E69" s="22" t="s">
-        <v>55</v>
+      <c r="D69" s="19" t="s">
+        <v>21</v>
       </c>
+      <c r="E69" s="10"/>
       <c r="F69" s="4"/>
       <c r="G69" s="4"/>
       <c r="H69" s="4"/>
@@ -3008,14 +3009,16 @@
     </row>
     <row r="70">
       <c r="A70" s="18" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B70" s="17">
         <v>1.0</v>
       </c>
       <c r="C70" s="4"/>
       <c r="D70" s="19"/>
-      <c r="E70" s="10"/>
+      <c r="E70" s="22" t="s">
+        <v>56</v>
+      </c>
       <c r="F70" s="4"/>
       <c r="G70" s="4"/>
       <c r="H70" s="4"/>
@@ -3047,9 +3050,7 @@
       </c>
       <c r="C71" s="4"/>
       <c r="D71" s="19"/>
-      <c r="E71" s="22" t="s">
-        <v>55</v>
-      </c>
+      <c r="E71" s="10"/>
       <c r="F71" s="4"/>
       <c r="G71" s="4"/>
       <c r="H71" s="4"/>
@@ -3081,7 +3082,9 @@
       </c>
       <c r="C72" s="4"/>
       <c r="D72" s="19"/>
-      <c r="E72" s="10"/>
+      <c r="E72" s="22" t="s">
+        <v>56</v>
+      </c>
       <c r="F72" s="4"/>
       <c r="G72" s="4"/>
       <c r="H72" s="4"/>
@@ -3105,16 +3108,14 @@
       <c r="Z72" s="4"/>
     </row>
     <row r="73">
-      <c r="A73" s="9" t="s">
+      <c r="A73" s="18" t="s">
         <v>59</v>
       </c>
       <c r="B73" s="17">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="C73" s="4"/>
-      <c r="D73" s="19" t="s">
-        <v>21</v>
-      </c>
+      <c r="D73" s="19"/>
       <c r="E73" s="10"/>
       <c r="F73" s="4"/>
       <c r="G73" s="4"/>
@@ -3143,10 +3144,10 @@
         <v>60</v>
       </c>
       <c r="B74" s="17">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="C74" s="4"/>
-      <c r="D74" s="21" t="s">
+      <c r="D74" s="19" t="s">
         <v>21</v>
       </c>
       <c r="E74" s="10"/>
@@ -3173,14 +3174,16 @@
       <c r="Z74" s="4"/>
     </row>
     <row r="75">
-      <c r="A75" s="18" t="s">
+      <c r="A75" s="9" t="s">
         <v>61</v>
       </c>
       <c r="B75" s="17">
         <v>1.0</v>
       </c>
       <c r="C75" s="4"/>
-      <c r="D75" s="29"/>
+      <c r="D75" s="21" t="s">
+        <v>21</v>
+      </c>
       <c r="E75" s="10"/>
       <c r="F75" s="4"/>
       <c r="G75" s="4"/>
@@ -3212,9 +3215,7 @@
         <v>1.0</v>
       </c>
       <c r="C76" s="4"/>
-      <c r="D76" s="21" t="s">
-        <v>21</v>
-      </c>
+      <c r="D76" s="29"/>
       <c r="E76" s="10"/>
       <c r="F76" s="4"/>
       <c r="G76" s="4"/>
@@ -3239,19 +3240,17 @@
       <c r="Z76" s="4"/>
     </row>
     <row r="77">
-      <c r="A77" s="9" t="s">
+      <c r="A77" s="18" t="s">
         <v>63</v>
       </c>
       <c r="B77" s="17">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="C77" s="4"/>
-      <c r="D77" s="19" t="s">
+      <c r="D77" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="E77" s="22" t="s">
-        <v>64</v>
-      </c>
+      <c r="E77" s="10"/>
       <c r="F77" s="4"/>
       <c r="G77" s="4"/>
       <c r="H77" s="4"/>
@@ -3275,11 +3274,19 @@
       <c r="Z77" s="4"/>
     </row>
     <row r="78">
-      <c r="A78" s="23"/>
-      <c r="B78" s="24"/>
-      <c r="C78" s="24"/>
-      <c r="D78" s="24"/>
-      <c r="E78" s="25"/>
+      <c r="A78" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B78" s="17">
+        <v>2.0</v>
+      </c>
+      <c r="C78" s="4"/>
+      <c r="D78" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="E78" s="22" t="s">
+        <v>65</v>
+      </c>
       <c r="F78" s="4"/>
       <c r="G78" s="4"/>
       <c r="H78" s="4"/>
@@ -3303,21 +3310,11 @@
       <c r="Z78" s="4"/>
     </row>
     <row r="79">
-      <c r="A79" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="B79" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="C79" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="D79" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="E79" s="16" t="s">
-        <v>11</v>
-      </c>
+      <c r="A79" s="23"/>
+      <c r="B79" s="24"/>
+      <c r="C79" s="24"/>
+      <c r="D79" s="24"/>
+      <c r="E79" s="25"/>
       <c r="F79" s="4"/>
       <c r="G79" s="4"/>
       <c r="H79" s="4"/>
@@ -3341,15 +3338,21 @@
       <c r="Z79" s="4"/>
     </row>
     <row r="80">
-      <c r="A80" s="9" t="s">
-        <v>12</v>
+      <c r="A80" s="28" t="s">
+        <v>66</v>
       </c>
-      <c r="B80" s="17">
-        <v>4.0</v>
+      <c r="B80" s="14" t="s">
+        <v>8</v>
       </c>
-      <c r="C80" s="4"/>
-      <c r="D80" s="4"/>
-      <c r="E80" s="10"/>
+      <c r="C80" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D80" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E80" s="16" t="s">
+        <v>11</v>
+      </c>
       <c r="F80" s="4"/>
       <c r="G80" s="4"/>
       <c r="H80" s="4"/>
@@ -3374,10 +3377,10 @@
     </row>
     <row r="81">
       <c r="A81" s="9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B81" s="17">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="C81" s="4"/>
       <c r="D81" s="4"/>
@@ -3406,10 +3409,10 @@
     </row>
     <row r="82">
       <c r="A82" s="9" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="B82" s="17">
-        <v>5.0</v>
+        <v>1.0</v>
       </c>
       <c r="C82" s="4"/>
       <c r="D82" s="4"/>
@@ -3438,10 +3441,10 @@
     </row>
     <row r="83">
       <c r="A83" s="9" t="s">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="B83" s="17">
-        <v>1.0</v>
+        <v>5.0</v>
       </c>
       <c r="C83" s="4"/>
       <c r="D83" s="4"/>
@@ -3473,7 +3476,7 @@
         <v>67</v>
       </c>
       <c r="B84" s="17">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="C84" s="4"/>
       <c r="D84" s="4"/>
@@ -3505,7 +3508,7 @@
         <v>68</v>
       </c>
       <c r="B85" s="17">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="C85" s="4"/>
       <c r="D85" s="4"/>
@@ -3540,7 +3543,7 @@
         <v>4.0</v>
       </c>
       <c r="C86" s="4"/>
-      <c r="D86" s="19"/>
+      <c r="D86" s="4"/>
       <c r="E86" s="10"/>
       <c r="F86" s="4"/>
       <c r="G86" s="4"/>
@@ -3566,13 +3569,13 @@
     </row>
     <row r="87">
       <c r="A87" s="9" t="s">
-        <v>23</v>
+        <v>70</v>
       </c>
       <c r="B87" s="17">
         <v>4.0</v>
       </c>
       <c r="C87" s="4"/>
-      <c r="D87" s="4"/>
+      <c r="D87" s="19"/>
       <c r="E87" s="10"/>
       <c r="F87" s="4"/>
       <c r="G87" s="4"/>
@@ -3598,10 +3601,10 @@
     </row>
     <row r="88">
       <c r="A88" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B88" s="17">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="C88" s="4"/>
       <c r="D88" s="4"/>
@@ -3630,15 +3633,13 @@
     </row>
     <row r="89">
       <c r="A89" s="9" t="s">
-        <v>70</v>
+        <v>24</v>
       </c>
       <c r="B89" s="17">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="C89" s="4"/>
-      <c r="D89" s="19" t="s">
-        <v>21</v>
-      </c>
+      <c r="D89" s="4"/>
       <c r="E89" s="10"/>
       <c r="F89" s="4"/>
       <c r="G89" s="4"/>
@@ -3669,9 +3670,7 @@
       <c r="B90" s="17">
         <v>1.0</v>
       </c>
-      <c r="C90" s="4" t="s">
-        <v>72</v>
-      </c>
+      <c r="C90" s="4"/>
       <c r="D90" s="19" t="s">
         <v>21</v>
       </c>
@@ -3699,21 +3698,19 @@
       <c r="Z90" s="4"/>
     </row>
     <row r="91">
-      <c r="A91" s="18" t="s">
-        <v>73</v>
+      <c r="A91" s="9" t="s">
+        <v>72</v>
       </c>
       <c r="B91" s="17">
         <v>1.0</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
-      <c r="D91" s="21" t="s">
+      <c r="D91" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="E91" s="22" t="s">
-        <v>75</v>
-      </c>
+      <c r="E91" s="10"/>
       <c r="F91" s="4"/>
       <c r="G91" s="4"/>
       <c r="H91" s="4"/>
@@ -3738,18 +3735,20 @@
     </row>
     <row r="92">
       <c r="A92" s="18" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B92" s="17">
         <v>1.0</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
-      <c r="D92" s="19" t="s">
+      <c r="D92" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="E92" s="10"/>
+      <c r="E92" s="22" t="s">
+        <v>76</v>
+      </c>
       <c r="F92" s="4"/>
       <c r="G92" s="4"/>
       <c r="H92" s="4"/>
@@ -3773,11 +3772,19 @@
       <c r="Z92" s="4"/>
     </row>
     <row r="93">
-      <c r="A93" s="23"/>
-      <c r="B93" s="24"/>
-      <c r="C93" s="24"/>
-      <c r="D93" s="24"/>
-      <c r="E93" s="25"/>
+      <c r="A93" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="B93" s="17">
+        <v>1.0</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D93" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="E93" s="10"/>
       <c r="F93" s="4"/>
       <c r="G93" s="4"/>
       <c r="H93" s="4"/>
@@ -3801,21 +3808,11 @@
       <c r="Z93" s="4"/>
     </row>
     <row r="94">
-      <c r="A94" s="30" t="s">
-        <v>78</v>
-      </c>
-      <c r="B94" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="C94" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="D94" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="E94" s="16" t="s">
-        <v>11</v>
-      </c>
+      <c r="A94" s="23"/>
+      <c r="B94" s="24"/>
+      <c r="C94" s="24"/>
+      <c r="D94" s="24"/>
+      <c r="E94" s="25"/>
       <c r="F94" s="4"/>
       <c r="G94" s="4"/>
       <c r="H94" s="4"/>
@@ -3839,18 +3836,20 @@
       <c r="Z94" s="4"/>
     </row>
     <row r="95">
-      <c r="A95" s="9" t="s">
+      <c r="A95" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="B95" s="31">
-        <v>1.0</v>
+      <c r="B95" s="14" t="s">
+        <v>8</v>
       </c>
-      <c r="C95" s="4" t="s">
-        <v>80</v>
+      <c r="C95" s="15" t="s">
+        <v>9</v>
       </c>
-      <c r="D95" s="4"/>
-      <c r="E95" s="22" t="s">
-        <v>81</v>
+      <c r="D95" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E95" s="16" t="s">
+        <v>11</v>
       </c>
       <c r="F95" s="4"/>
       <c r="G95" s="4"/>
@@ -3876,16 +3875,18 @@
     </row>
     <row r="96">
       <c r="A96" s="9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B96" s="31">
         <v>1.0</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D96" s="4"/>
-      <c r="E96" s="10"/>
+      <c r="E96" s="22" t="s">
+        <v>82</v>
+      </c>
       <c r="F96" s="4"/>
       <c r="G96" s="4"/>
       <c r="H96" s="4"/>
@@ -3910,18 +3911,16 @@
     </row>
     <row r="97">
       <c r="A97" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B97" s="31">
         <v>1.0</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D97" s="4"/>
-      <c r="E97" s="10" t="s">
-        <v>81</v>
-      </c>
+      <c r="E97" s="10"/>
       <c r="F97" s="4"/>
       <c r="G97" s="4"/>
       <c r="H97" s="4"/>
@@ -3945,11 +3944,19 @@
       <c r="Z97" s="4"/>
     </row>
     <row r="98">
-      <c r="A98" s="23"/>
-      <c r="B98" s="24"/>
-      <c r="C98" s="24"/>
-      <c r="D98" s="24"/>
-      <c r="E98" s="25"/>
+      <c r="A98" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="B98" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D98" s="4"/>
+      <c r="E98" s="10" t="s">
+        <v>82</v>
+      </c>
       <c r="F98" s="4"/>
       <c r="G98" s="4"/>
       <c r="H98" s="4"/>
@@ -3973,11 +3980,11 @@
       <c r="Z98" s="4"/>
     </row>
     <row r="99">
-      <c r="A99" s="4"/>
-      <c r="B99" s="4"/>
-      <c r="C99" s="4"/>
-      <c r="D99" s="4"/>
-      <c r="E99" s="4"/>
+      <c r="A99" s="23"/>
+      <c r="B99" s="24"/>
+      <c r="C99" s="24"/>
+      <c r="D99" s="24"/>
+      <c r="E99" s="25"/>
       <c r="F99" s="4"/>
       <c r="G99" s="4"/>
       <c r="H99" s="4"/>
@@ -29872,6 +29879,34 @@
       <c r="Y1023" s="4"/>
       <c r="Z1023" s="4"/>
     </row>
+    <row r="1024">
+      <c r="A1024" s="4"/>
+      <c r="B1024" s="4"/>
+      <c r="C1024" s="4"/>
+      <c r="D1024" s="4"/>
+      <c r="E1024" s="4"/>
+      <c r="F1024" s="4"/>
+      <c r="G1024" s="4"/>
+      <c r="H1024" s="4"/>
+      <c r="I1024" s="4"/>
+      <c r="J1024" s="4"/>
+      <c r="K1024" s="4"/>
+      <c r="L1024" s="4"/>
+      <c r="M1024" s="4"/>
+      <c r="N1024" s="4"/>
+      <c r="O1024" s="4"/>
+      <c r="P1024" s="4"/>
+      <c r="Q1024" s="4"/>
+      <c r="R1024" s="4"/>
+      <c r="S1024" s="4"/>
+      <c r="T1024" s="4"/>
+      <c r="U1024" s="4"/>
+      <c r="V1024" s="4"/>
+      <c r="W1024" s="4"/>
+      <c r="X1024" s="4"/>
+      <c r="Y1024" s="4"/>
+      <c r="Z1024" s="4"/>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:E1"/>
@@ -29895,16 +29930,16 @@
     <hyperlink r:id="rId11" ref="D46"/>
     <hyperlink r:id="rId12" ref="D47"/>
     <hyperlink r:id="rId13" ref="D48"/>
-    <hyperlink r:id="rId14" ref="D65"/>
-    <hyperlink r:id="rId15" ref="D68"/>
-    <hyperlink r:id="rId16" ref="D73"/>
-    <hyperlink r:id="rId17" ref="D74"/>
-    <hyperlink r:id="rId18" ref="D76"/>
-    <hyperlink r:id="rId19" ref="D77"/>
-    <hyperlink r:id="rId20" ref="D89"/>
-    <hyperlink r:id="rId21" ref="D90"/>
-    <hyperlink r:id="rId22" ref="D91"/>
-    <hyperlink r:id="rId23" ref="D92"/>
+    <hyperlink r:id="rId14" ref="D66"/>
+    <hyperlink r:id="rId15" ref="D69"/>
+    <hyperlink r:id="rId16" ref="D74"/>
+    <hyperlink r:id="rId17" ref="D75"/>
+    <hyperlink r:id="rId18" ref="D77"/>
+    <hyperlink r:id="rId19" ref="D78"/>
+    <hyperlink r:id="rId20" ref="D90"/>
+    <hyperlink r:id="rId21" ref="D91"/>
+    <hyperlink r:id="rId22" ref="D92"/>
+    <hyperlink r:id="rId23" ref="D93"/>
   </hyperlinks>
   <drawing r:id="rId24"/>
 </worksheet>

</xml_diff>